<commit_message>
Solved example: every messy label now visible (silent flr), cleaning log gives before/after, how it was spotted and why, blank cells marked; workbook updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FbSp4cD9x3d7McJz35Da8q
</commit_message>
<xml_diff>
--- a/assets/charts/GED106_Week9_Solved_Example.xlsx
+++ b/assets/charts/GED106_Week9_Solved_Example.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="110">
   <si>
     <t xml:space="preserve">Solved example · Library study spaces survey</t>
   </si>
@@ -185,7 +185,7 @@
     <t xml:space="preserve">Café corner</t>
   </si>
   <si>
-    <t xml:space="preserve">Silent  floor</t>
+    <t xml:space="preserve">silent flr</t>
   </si>
   <si>
     <t xml:space="preserve">More power sockets</t>
@@ -209,13 +209,16 @@
     <t xml:space="preserve">Issue</t>
   </si>
   <si>
-    <t xml:space="preserve">Rows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What I did</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Why</t>
+    <t xml:space="preserve">Row</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Before → After</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How I spotted it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Why this fix</t>
   </si>
   <si>
     <t xml:space="preserve">Test row</t>
@@ -224,43 +227,97 @@
     <t xml:space="preserve">ID 0</t>
   </si>
   <si>
-    <t xml:space="preserve">Deleted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not a real student</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Duplicates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IDs 6 and 20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Removed the extra copy (Data → Remove Duplicates)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Each student counts once</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Labels</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IDs 4, 9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">“year 2”, “2nd year” → Year 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same answer, different spelling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IDs 13, 17, 22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">“Silent  floor”, “group rooms”, “Computers” → Silent floor, Group rooms, Computer area</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same category, different spelling</t>
+    <t xml:space="preserve">“TEST - ignore” → row deleted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The ID is 0 and the answer says “TEST”: it was the form owner checking the survey.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">It is not a real student, so it would change every count.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duplicate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two identical rows → one kept</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sort by ID: ID 6 appears twice with exactly the same answers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One student must count once; a copy inflates the counts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same check: ID 20 appears twice. Data → Remove Duplicates on ID.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same reason: each response counts once.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inconsistent label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“year 2” → Year 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filter the Year column: “year 2” shows as a separate option.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excel counts “year 2” and “Year 2” as different groups unless they match exactly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID 9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“2nd year” → Year 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same filter: “2nd year” is the same answer written another way.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All answers must use the form’s options: Year 1, Year 2, Year 3, Year 4+.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“silent flr” → Silent floor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filter the Space column: “silent flr” is a typing variant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Otherwise Silent floor is under-counted by one.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID 17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“group rooms” → Group rooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same filter: lower-case variant of an option.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same reason: one category, one spelling.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID 22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“Computers” → Computer area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same filter: a shortened name of an option.</t>
   </si>
   <si>
     <t xml:space="preserve">Impossible value</t>
@@ -272,7 +329,10 @@
     <t xml:space="preserve">Rating 6 → blank</t>
   </si>
   <si>
-    <t xml:space="preserve">Outside the 1–5 scale</t>
+    <t xml:space="preserve">Filter Satisfaction: the scale is 1–5, so 6 cannot be a real answer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We cannot know the true rating, so we remove it instead of changing it to 5.</t>
   </si>
   <si>
     <t xml:space="preserve">Missing value</t>
@@ -281,10 +341,13 @@
     <t xml:space="preserve">ID 19</t>
   </si>
   <si>
-    <t xml:space="preserve">Hours left blank, not guessed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Guessing adds false data</t>
+    <t xml:space="preserve">Hours: blank → left blank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filter Hours: one empty cell.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Never guess: an invented value is false data. COUNTIF simply skips the blank.</t>
   </si>
   <si>
     <t xml:space="preserve">Students</t>
@@ -671,11 +734,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="46176006"/>
-        <c:axId val="5868931"/>
+        <c:axId val="69492080"/>
+        <c:axId val="53859988"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="46176006"/>
+        <c:axId val="69492080"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -741,7 +804,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5868931"/>
+        <c:crossAx val="53859988"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -749,7 +812,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="5868931"/>
+        <c:axId val="53859988"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -825,7 +888,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46176006"/>
+        <c:crossAx val="69492080"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -985,11 +1048,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="72798937"/>
-        <c:axId val="19472192"/>
+        <c:axId val="12935234"/>
+        <c:axId val="24961009"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="72798937"/>
+        <c:axId val="12935234"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1055,7 +1118,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19472192"/>
+        <c:crossAx val="24961009"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1063,7 +1126,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="19472192"/>
+        <c:axId val="24961009"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1139,7 +1202,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="72798937"/>
+        <c:crossAx val="12935234"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2955,12 +3018,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="44"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2976,89 +3040,178 @@
       <c r="D1" s="3" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E1" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C3" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="B4" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>74</v>
-      </c>
       <c r="D4" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>79</v>
-      </c>
       <c r="B6" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>85</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -3092,13 +3245,13 @@
         <v>32</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>88</v>
+        <v>109</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>